<commit_message>
Update plots and tables
</commit_message>
<xml_diff>
--- a/Tables/CAAR.xlsx
+++ b/Tables/CAAR.xlsx
@@ -470,19 +470,19 @@
         <v>-0.115787711999745</v>
       </c>
       <c r="C2" t="n">
-        <v>-0.003653582663624462</v>
+        <v>0.01335354411790846</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.00196625161560518</v>
+        <v>-0.004586483754647954</v>
       </c>
       <c r="E2" t="n">
-        <v>-1.918316325774458</v>
+        <v>-1.893016925295929</v>
       </c>
       <c r="F2" t="n">
-        <v>1.921926267478224</v>
+        <v>1.953648726493962</v>
       </c>
       <c r="G2" t="n">
-        <v>0.9064</v>
+        <v>0.9069</v>
       </c>
     </row>
     <row r="3">
@@ -495,19 +495,19 @@
         <v>-1.182483644484863</v>
       </c>
       <c r="C3" t="n">
-        <v>-0.007229108989866388</v>
+        <v>0.008068347476074397</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.02157847145322379</v>
+        <v>-0.004073508082171107</v>
       </c>
       <c r="E3" t="n">
-        <v>-1.544448164649104</v>
+        <v>-1.549535193961144</v>
       </c>
       <c r="F3" t="n">
-        <v>1.582824169947167</v>
+        <v>1.592756387339704</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1449</v>
+        <v>0.1473</v>
       </c>
     </row>
     <row r="4">
@@ -517,22 +517,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.7369935532877838</v>
+        <v>-0.8798423933694248</v>
       </c>
       <c r="C4" t="n">
-        <v>-0.00381580439292437</v>
+        <v>0.01494210236098054</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.003312215925577594</v>
+        <v>0.005921086528211016</v>
       </c>
       <c r="E4" t="n">
-        <v>-2.252272351261925</v>
+        <v>-1.92307259479026</v>
       </c>
       <c r="F4" t="n">
-        <v>2.183904256126337</v>
+        <v>1.986870752199494</v>
       </c>
       <c r="G4" t="n">
-        <v>0.5158</v>
+        <v>0.375</v>
       </c>
     </row>
     <row r="5">
@@ -542,22 +542,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.4474648098159981</v>
+        <v>-0.5903136498976391</v>
       </c>
       <c r="C5" t="n">
-        <v>0.008171336215119217</v>
+        <v>0.009334840989667581</v>
       </c>
       <c r="D5" t="n">
-        <v>0.02114672619897275</v>
+        <v>-0.003549965971851171</v>
       </c>
       <c r="E5" t="n">
-        <v>-2.738021529154462</v>
+        <v>-2.463106056520016</v>
       </c>
       <c r="F5" t="n">
-        <v>2.746697430324348</v>
+        <v>2.560204426954504</v>
       </c>
       <c r="G5" t="n">
-        <v>0.7479</v>
+        <v>0.6389</v>
       </c>
     </row>
   </sheetData>

</xml_diff>